<commit_message>
Dashboard en cm, pestaña Caja por caja y lectura de un tratamiento por columna
</commit_message>
<xml_diff>
--- a/Tiempo_30 s.xlsx
+++ b/Tiempo_30 s.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e77740388cd245da/Imágenes/pred/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e77740388cd245da/Documentos/chat/BioGrow/dashboard_semillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA96AB9-35D3-44D1-84EF-0844202AB554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3780" yWindow="1710" windowWidth="17940" windowHeight="9360" xr2:uid="{650DD92F-AD60-4C65-89EA-E431E3430616}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{650DD92F-AD60-4C65-89EA-E431E3430616}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>